<commit_message>
Peripherals Added in BOM.
</commit_message>
<xml_diff>
--- a/Design-Files/BOM/Royluo-Client-BOM.xlsx
+++ b/Design-Files/BOM/Royluo-Client-BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\royluo-ledboard\Design-Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1844785-CB95-4D23-82C0-F2E88CC111E5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27671CC4-12F1-4FEA-AA20-00547A57FD5E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="84">
   <si>
     <t>#</t>
   </si>
@@ -260,13 +260,25 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Alibaba</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>Coin Cell CR1220</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -309,6 +321,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -422,10 +442,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -465,8 +486,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -752,7 +777,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -971,7 +996,9 @@
       <c r="J7" s="7">
         <v>1</v>
       </c>
-      <c r="K7" s="7"/>
+      <c r="K7" s="15" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1200,7 +1227,6 @@
     <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
-        <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
@@ -1228,12 +1254,50 @@
         <v>1</v>
       </c>
       <c r="K15" s="7"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1"/>
+      <c r="B16" s="11">
+        <f>ROW(B16) - ROW($B$2)</f>
+        <v>14</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="J16" s="7">
+        <v>2</v>
+      </c>
+      <c r="K16" s="15" t="s">
+        <v>83</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K7" r:id="rId1" xr:uid="{26AE188D-ED6F-4273-A1EF-393FBCA89064}"/>
+    <hyperlink ref="K16" r:id="rId2" xr:uid="{364EDEA2-FF0B-4A17-8E98-C01DBB29BCA1}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>